<commit_message>
chuan bi cho xuat ca
</commit_message>
<xml_diff>
--- a/data1.xlsx
+++ b/data1.xlsx
@@ -289,9 +289,6 @@
     <t>7.0</t>
   </si>
   <si>
-    <t>RR5</t>
-  </si>
-  <si>
     <t>2021-01-10</t>
   </si>
   <si>
@@ -446,6 +443,9 @@
   </si>
   <si>
     <t>07:30</t>
+  </si>
+  <si>
+    <t>NT7</t>
   </si>
   <si>
     <t>11:30</t>
@@ -1800,7 +1800,7 @@
         <v>0</v>
       </c>
       <c r="AK12" t="s">
-        <v>91</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -1814,7 +1814,7 @@
         <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E13" t="s">
         <v>64</v>
@@ -1835,7 +1835,7 @@
         <v>44</v>
       </c>
       <c r="M13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N13" t="s">
         <v>88</v>
@@ -1903,7 +1903,7 @@
         <v>40</v>
       </c>
       <c r="D14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E14" t="s">
         <v>70</v>
@@ -1995,7 +1995,7 @@
         <v>40</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E15" t="s">
         <v>72</v>
@@ -2022,22 +2022,22 @@
         <v>59</v>
       </c>
       <c r="N15" t="s">
+        <v>95</v>
+      </c>
+      <c r="O15" t="s">
+        <v>95</v>
+      </c>
+      <c r="P15" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>48</v>
+      </c>
+      <c r="T15" t="s">
         <v>96</v>
       </c>
-      <c r="O15" t="s">
+      <c r="U15" t="s">
         <v>96</v>
-      </c>
-      <c r="P15" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>48</v>
-      </c>
-      <c r="T15" t="s">
-        <v>97</v>
-      </c>
-      <c r="U15" t="s">
-        <v>97</v>
       </c>
       <c r="V15" t="s">
         <v>51</v>
@@ -2052,7 +2052,7 @@
         <v>51</v>
       </c>
       <c r="AB15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AC15" t="s">
         <v>51</v>
@@ -2093,7 +2093,7 @@
         <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E16" t="s">
         <v>78</v>
@@ -2117,7 +2117,7 @@
         <v>44</v>
       </c>
       <c r="M16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="N16" t="s">
         <v>74</v>
@@ -2191,7 +2191,7 @@
         <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E17" t="s">
         <v>80</v>
@@ -2215,7 +2215,7 @@
         <v>44</v>
       </c>
       <c r="M17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N17" t="s">
         <v>86</v>
@@ -2239,7 +2239,7 @@
         <v>51</v>
       </c>
       <c r="Y17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Z17" t="s">
         <v>53</v>
@@ -2254,7 +2254,7 @@
         <v>51</v>
       </c>
       <c r="AD17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AE17" t="s">
         <v>51</v>
@@ -2289,7 +2289,7 @@
         <v>40</v>
       </c>
       <c r="D18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E18" t="s">
         <v>42</v>
@@ -2384,7 +2384,7 @@
         <v>40</v>
       </c>
       <c r="D19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E19" t="s">
         <v>57</v>
@@ -2408,13 +2408,13 @@
         <v>44</v>
       </c>
       <c r="M19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P19" t="s">
         <v>48</v>
@@ -2479,7 +2479,7 @@
         <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E20" t="s">
         <v>64</v>
@@ -2500,7 +2500,7 @@
         <v>44</v>
       </c>
       <c r="M20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N20" t="s">
         <v>67</v>
@@ -2568,7 +2568,7 @@
         <v>40</v>
       </c>
       <c r="D21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E21" t="s">
         <v>70</v>
@@ -2663,7 +2663,7 @@
         <v>40</v>
       </c>
       <c r="D22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E22" t="s">
         <v>72</v>
@@ -2687,13 +2687,13 @@
         <v>44</v>
       </c>
       <c r="M22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="N22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P22" t="s">
         <v>48</v>
@@ -2758,7 +2758,7 @@
         <v>40</v>
       </c>
       <c r="D23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E23" t="s">
         <v>78</v>
@@ -2782,13 +2782,13 @@
         <v>44</v>
       </c>
       <c r="M23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="N23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P23" t="s">
         <v>48</v>
@@ -2797,10 +2797,10 @@
         <v>48</v>
       </c>
       <c r="T23" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="U23" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="V23" t="s">
         <v>51</v>
@@ -2853,7 +2853,7 @@
         <v>40</v>
       </c>
       <c r="D24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E24" t="s">
         <v>80</v>
@@ -2948,7 +2948,7 @@
         <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E25" t="s">
         <v>42</v>
@@ -3043,7 +3043,7 @@
         <v>40</v>
       </c>
       <c r="D26" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E26" t="s">
         <v>57</v>
@@ -3138,7 +3138,7 @@
         <v>40</v>
       </c>
       <c r="D27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E27" t="s">
         <v>64</v>
@@ -3215,7 +3215,7 @@
         <v>40</v>
       </c>
       <c r="D28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E28" t="s">
         <v>70</v>
@@ -3310,7 +3310,7 @@
         <v>40</v>
       </c>
       <c r="D29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E29" t="s">
         <v>72</v>
@@ -3405,7 +3405,7 @@
         <v>40</v>
       </c>
       <c r="D30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E30" t="s">
         <v>78</v>
@@ -3500,7 +3500,7 @@
         <v>40</v>
       </c>
       <c r="D31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E31" t="s">
         <v>80</v>
@@ -3595,7 +3595,7 @@
         <v>40</v>
       </c>
       <c r="D32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E32" t="s">
         <v>42</v>
@@ -3690,7 +3690,7 @@
         <v>40</v>
       </c>
       <c r="D33" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E33" t="s">
         <v>57</v>
@@ -3785,7 +3785,7 @@
         <v>40</v>
       </c>
       <c r="D34" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E34" t="s">
         <v>64</v>
@@ -3806,7 +3806,7 @@
         <v>74</v>
       </c>
       <c r="M34" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N34" t="s">
         <v>58</v>
@@ -3842,7 +3842,7 @@
         <v>51</v>
       </c>
       <c r="AE34" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AF34" t="s">
         <v>51</v>
@@ -3865,10 +3865,10 @@
     </row>
     <row r="35" spans="1:37">
       <c r="A35" t="s">
+        <v>123</v>
+      </c>
+      <c r="B35" t="s">
         <v>124</v>
-      </c>
-      <c r="B35" t="s">
-        <v>125</v>
       </c>
       <c r="C35" t="s">
         <v>40</v>
@@ -3880,7 +3880,7 @@
         <v>42</v>
       </c>
       <c r="F35" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G35" t="s">
         <v>45</v>
@@ -3916,7 +3916,7 @@
         <v>52</v>
       </c>
       <c r="Z35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AA35" t="s">
         <v>51</v>
@@ -3954,10 +3954,10 @@
     </row>
     <row r="36" spans="1:37">
       <c r="A36" t="s">
+        <v>123</v>
+      </c>
+      <c r="B36" t="s">
         <v>124</v>
-      </c>
-      <c r="B36" t="s">
-        <v>125</v>
       </c>
       <c r="C36" t="s">
         <v>40</v>
@@ -3969,7 +3969,7 @@
         <v>57</v>
       </c>
       <c r="F36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G36" t="s">
         <v>45</v>
@@ -4008,7 +4008,7 @@
         <v>58</v>
       </c>
       <c r="Z36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA36" t="s">
         <v>51</v>
@@ -4041,15 +4041,15 @@
         <v>0</v>
       </c>
       <c r="AK36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="37" spans="1:37">
       <c r="A37" t="s">
+        <v>123</v>
+      </c>
+      <c r="B37" t="s">
         <v>124</v>
-      </c>
-      <c r="B37" t="s">
-        <v>125</v>
       </c>
       <c r="C37" t="s">
         <v>40</v>
@@ -4073,7 +4073,7 @@
         <v>47</v>
       </c>
       <c r="L37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M37" t="s">
         <v>48</v>
@@ -4126,10 +4126,10 @@
     </row>
     <row r="38" spans="1:37">
       <c r="A38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B38" t="s">
         <v>124</v>
-      </c>
-      <c r="B38" t="s">
-        <v>125</v>
       </c>
       <c r="C38" t="s">
         <v>40</v>
@@ -4141,7 +4141,7 @@
         <v>70</v>
       </c>
       <c r="F38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G38" t="s">
         <v>45</v>
@@ -4177,7 +4177,7 @@
         <v>51</v>
       </c>
       <c r="Z38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA38" t="s">
         <v>51</v>
@@ -4210,15 +4210,15 @@
         <v>0</v>
       </c>
       <c r="AK38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:37">
       <c r="A39" t="s">
+        <v>123</v>
+      </c>
+      <c r="B39" t="s">
         <v>124</v>
-      </c>
-      <c r="B39" t="s">
-        <v>125</v>
       </c>
       <c r="C39" t="s">
         <v>40</v>
@@ -4230,7 +4230,7 @@
         <v>72</v>
       </c>
       <c r="F39" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G39" t="s">
         <v>45</v>
@@ -4245,7 +4245,7 @@
         <v>47</v>
       </c>
       <c r="L39" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M39" t="s">
         <v>44</v>
@@ -4266,10 +4266,10 @@
         <v>51</v>
       </c>
       <c r="Y39" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Z39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AA39" t="s">
         <v>47</v>
@@ -4302,15 +4302,15 @@
         <v>0</v>
       </c>
       <c r="AK39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:37">
       <c r="A40" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" t="s">
         <v>124</v>
-      </c>
-      <c r="B40" t="s">
-        <v>125</v>
       </c>
       <c r="C40" t="s">
         <v>40</v>
@@ -4322,7 +4322,7 @@
         <v>78</v>
       </c>
       <c r="F40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G40" t="s">
         <v>45</v>
@@ -4358,7 +4358,7 @@
         <v>52</v>
       </c>
       <c r="Z40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AA40" t="s">
         <v>51</v>
@@ -4396,10 +4396,10 @@
     </row>
     <row r="41" spans="1:37">
       <c r="A41" t="s">
+        <v>123</v>
+      </c>
+      <c r="B41" t="s">
         <v>124</v>
-      </c>
-      <c r="B41" t="s">
-        <v>125</v>
       </c>
       <c r="C41" t="s">
         <v>40</v>
@@ -4411,7 +4411,7 @@
         <v>80</v>
       </c>
       <c r="F41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G41" t="s">
         <v>45</v>
@@ -4447,7 +4447,7 @@
         <v>84</v>
       </c>
       <c r="Z41" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AA41" t="s">
         <v>51</v>
@@ -4485,10 +4485,10 @@
     </row>
     <row r="42" spans="1:37">
       <c r="A42" t="s">
+        <v>123</v>
+      </c>
+      <c r="B42" t="s">
         <v>124</v>
-      </c>
-      <c r="B42" t="s">
-        <v>125</v>
       </c>
       <c r="C42" t="s">
         <v>40</v>
@@ -4500,7 +4500,7 @@
         <v>42</v>
       </c>
       <c r="F42" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G42" t="s">
         <v>45</v>
@@ -4518,7 +4518,7 @@
         <v>45</v>
       </c>
       <c r="M42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N42" t="s">
         <v>88</v>
@@ -4572,15 +4572,15 @@
         <v>0</v>
       </c>
       <c r="AK42" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:37">
       <c r="A43" t="s">
+        <v>123</v>
+      </c>
+      <c r="B43" t="s">
         <v>124</v>
-      </c>
-      <c r="B43" t="s">
-        <v>125</v>
       </c>
       <c r="C43" t="s">
         <v>40</v>
@@ -4592,7 +4592,7 @@
         <v>57</v>
       </c>
       <c r="F43" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G43" t="s">
         <v>45</v>
@@ -4664,21 +4664,21 @@
         <v>0</v>
       </c>
       <c r="AK43" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:37">
       <c r="A44" t="s">
+        <v>123</v>
+      </c>
+      <c r="B44" t="s">
         <v>124</v>
-      </c>
-      <c r="B44" t="s">
-        <v>125</v>
       </c>
       <c r="C44" t="s">
         <v>40</v>
       </c>
       <c r="D44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E44" t="s">
         <v>64</v>
@@ -4749,22 +4749,22 @@
     </row>
     <row r="45" spans="1:37">
       <c r="A45" t="s">
+        <v>123</v>
+      </c>
+      <c r="B45" t="s">
         <v>124</v>
-      </c>
-      <c r="B45" t="s">
-        <v>125</v>
       </c>
       <c r="C45" t="s">
         <v>40</v>
       </c>
       <c r="D45" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E45" t="s">
         <v>70</v>
       </c>
       <c r="F45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G45" t="s">
         <v>45</v>
@@ -4800,7 +4800,7 @@
         <v>51</v>
       </c>
       <c r="Z45" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA45" t="s">
         <v>51</v>
@@ -4833,27 +4833,27 @@
         <v>0</v>
       </c>
       <c r="AK45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:37">
       <c r="A46" t="s">
+        <v>123</v>
+      </c>
+      <c r="B46" t="s">
         <v>124</v>
-      </c>
-      <c r="B46" t="s">
-        <v>125</v>
       </c>
       <c r="C46" t="s">
         <v>40</v>
       </c>
       <c r="D46" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E46" t="s">
         <v>72</v>
       </c>
       <c r="F46" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G46" t="s">
         <v>45</v>
@@ -4874,10 +4874,10 @@
         <v>88</v>
       </c>
       <c r="N46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P46" t="s">
         <v>48</v>
@@ -4889,7 +4889,7 @@
         <v>51</v>
       </c>
       <c r="Z46" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA46" t="s">
         <v>51</v>
@@ -4922,27 +4922,27 @@
         <v>0</v>
       </c>
       <c r="AK46" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:37">
       <c r="A47" t="s">
+        <v>123</v>
+      </c>
+      <c r="B47" t="s">
         <v>124</v>
-      </c>
-      <c r="B47" t="s">
-        <v>125</v>
       </c>
       <c r="C47" t="s">
         <v>40</v>
       </c>
       <c r="D47" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E47" t="s">
         <v>78</v>
       </c>
       <c r="F47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G47" t="s">
         <v>45</v>
@@ -4978,7 +4978,7 @@
         <v>51</v>
       </c>
       <c r="Z47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA47" t="s">
         <v>51</v>
@@ -5011,27 +5011,27 @@
         <v>0</v>
       </c>
       <c r="AK47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="48" spans="1:37">
       <c r="A48" t="s">
+        <v>123</v>
+      </c>
+      <c r="B48" t="s">
         <v>124</v>
-      </c>
-      <c r="B48" t="s">
-        <v>125</v>
       </c>
       <c r="C48" t="s">
         <v>40</v>
       </c>
       <c r="D48" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E48" t="s">
         <v>80</v>
       </c>
       <c r="F48" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G48" t="s">
         <v>45</v>
@@ -5052,10 +5052,10 @@
         <v>86</v>
       </c>
       <c r="N48" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O48" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P48" t="s">
         <v>48</v>
@@ -5067,7 +5067,7 @@
         <v>51</v>
       </c>
       <c r="Z48" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA48" t="s">
         <v>51</v>
@@ -5100,27 +5100,27 @@
         <v>0</v>
       </c>
       <c r="AK48" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:37">
       <c r="A49" t="s">
+        <v>123</v>
+      </c>
+      <c r="B49" t="s">
         <v>124</v>
-      </c>
-      <c r="B49" t="s">
-        <v>125</v>
       </c>
       <c r="C49" t="s">
         <v>40</v>
       </c>
       <c r="D49" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E49" t="s">
         <v>42</v>
       </c>
       <c r="F49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G49" t="s">
         <v>45</v>
@@ -5138,13 +5138,13 @@
         <v>45</v>
       </c>
       <c r="M49" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N49" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O49" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P49" t="s">
         <v>48</v>
@@ -5156,7 +5156,7 @@
         <v>51</v>
       </c>
       <c r="Z49" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AA49" t="s">
         <v>51</v>
@@ -5189,27 +5189,27 @@
         <v>0</v>
       </c>
       <c r="AK49" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:37">
       <c r="A50" t="s">
+        <v>123</v>
+      </c>
+      <c r="B50" t="s">
         <v>124</v>
-      </c>
-      <c r="B50" t="s">
-        <v>125</v>
       </c>
       <c r="C50" t="s">
         <v>40</v>
       </c>
       <c r="D50" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E50" t="s">
         <v>57</v>
       </c>
       <c r="F50" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G50" t="s">
         <v>45</v>
@@ -5289,16 +5289,16 @@
     </row>
     <row r="51" spans="1:37">
       <c r="A51" t="s">
+        <v>123</v>
+      </c>
+      <c r="B51" t="s">
         <v>124</v>
-      </c>
-      <c r="B51" t="s">
-        <v>125</v>
       </c>
       <c r="C51" t="s">
         <v>40</v>
       </c>
       <c r="D51" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E51" t="s">
         <v>64</v>
@@ -5355,7 +5355,7 @@
         <v>51</v>
       </c>
       <c r="AE51" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AF51" t="s">
         <v>51</v>
@@ -5378,22 +5378,22 @@
     </row>
     <row r="52" spans="1:37">
       <c r="A52" t="s">
+        <v>123</v>
+      </c>
+      <c r="B52" t="s">
         <v>124</v>
-      </c>
-      <c r="B52" t="s">
-        <v>125</v>
       </c>
       <c r="C52" t="s">
         <v>40</v>
       </c>
       <c r="D52" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E52" t="s">
         <v>70</v>
       </c>
       <c r="F52" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G52" t="s">
         <v>45</v>
@@ -5476,22 +5476,22 @@
     </row>
     <row r="53" spans="1:37">
       <c r="A53" t="s">
+        <v>123</v>
+      </c>
+      <c r="B53" t="s">
         <v>124</v>
-      </c>
-      <c r="B53" t="s">
-        <v>125</v>
       </c>
       <c r="C53" t="s">
         <v>40</v>
       </c>
       <c r="D53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E53" t="s">
         <v>72</v>
       </c>
       <c r="F53" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G53" t="s">
         <v>45</v>
@@ -5574,22 +5574,22 @@
     </row>
     <row r="54" spans="1:37">
       <c r="A54" t="s">
+        <v>123</v>
+      </c>
+      <c r="B54" t="s">
         <v>124</v>
-      </c>
-      <c r="B54" t="s">
-        <v>125</v>
       </c>
       <c r="C54" t="s">
         <v>40</v>
       </c>
       <c r="D54" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E54" t="s">
         <v>78</v>
       </c>
       <c r="F54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G54" t="s">
         <v>45</v>
@@ -5669,22 +5669,22 @@
     </row>
     <row r="55" spans="1:37">
       <c r="A55" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" t="s">
         <v>124</v>
-      </c>
-      <c r="B55" t="s">
-        <v>125</v>
       </c>
       <c r="C55" t="s">
         <v>40</v>
       </c>
       <c r="D55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E55" t="s">
         <v>80</v>
       </c>
       <c r="F55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G55" t="s">
         <v>45</v>
@@ -5764,22 +5764,22 @@
     </row>
     <row r="56" spans="1:37">
       <c r="A56" t="s">
+        <v>123</v>
+      </c>
+      <c r="B56" t="s">
         <v>124</v>
-      </c>
-      <c r="B56" t="s">
-        <v>125</v>
       </c>
       <c r="C56" t="s">
         <v>40</v>
       </c>
       <c r="D56" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E56" t="s">
         <v>42</v>
       </c>
       <c r="F56" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G56" t="s">
         <v>45</v>
@@ -5854,27 +5854,27 @@
         <v>4</v>
       </c>
       <c r="AK56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="57" spans="1:37">
       <c r="A57" t="s">
+        <v>123</v>
+      </c>
+      <c r="B57" t="s">
         <v>124</v>
-      </c>
-      <c r="B57" t="s">
-        <v>125</v>
       </c>
       <c r="C57" t="s">
         <v>40</v>
       </c>
       <c r="D57" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E57" t="s">
         <v>57</v>
       </c>
       <c r="F57" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G57" t="s">
         <v>45</v>
@@ -5949,21 +5949,21 @@
         <v>4</v>
       </c>
       <c r="AK57" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="58" spans="1:37">
       <c r="A58" t="s">
+        <v>123</v>
+      </c>
+      <c r="B58" t="s">
         <v>124</v>
-      </c>
-      <c r="B58" t="s">
-        <v>125</v>
       </c>
       <c r="C58" t="s">
         <v>40</v>
       </c>
       <c r="D58" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E58" t="s">
         <v>64</v>
@@ -6034,22 +6034,22 @@
     </row>
     <row r="59" spans="1:37">
       <c r="A59" t="s">
+        <v>123</v>
+      </c>
+      <c r="B59" t="s">
         <v>124</v>
-      </c>
-      <c r="B59" t="s">
-        <v>125</v>
       </c>
       <c r="C59" t="s">
         <v>40</v>
       </c>
       <c r="D59" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E59" t="s">
         <v>70</v>
       </c>
       <c r="F59" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G59" t="s">
         <v>45</v>
@@ -6124,27 +6124,27 @@
         <v>4</v>
       </c>
       <c r="AK59" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="60" spans="1:37">
       <c r="A60" t="s">
+        <v>123</v>
+      </c>
+      <c r="B60" t="s">
         <v>124</v>
-      </c>
-      <c r="B60" t="s">
-        <v>125</v>
       </c>
       <c r="C60" t="s">
         <v>40</v>
       </c>
       <c r="D60" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E60" t="s">
         <v>72</v>
       </c>
       <c r="F60" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G60" t="s">
         <v>45</v>
@@ -6219,27 +6219,27 @@
         <v>4</v>
       </c>
       <c r="AK60" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:37">
       <c r="A61" t="s">
+        <v>123</v>
+      </c>
+      <c r="B61" t="s">
         <v>124</v>
-      </c>
-      <c r="B61" t="s">
-        <v>125</v>
       </c>
       <c r="C61" t="s">
         <v>40</v>
       </c>
       <c r="D61" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E61" t="s">
         <v>78</v>
       </c>
       <c r="F61" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G61" t="s">
         <v>45</v>
@@ -6314,27 +6314,27 @@
         <v>4</v>
       </c>
       <c r="AK61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="62" spans="1:37">
       <c r="A62" t="s">
+        <v>123</v>
+      </c>
+      <c r="B62" t="s">
         <v>124</v>
-      </c>
-      <c r="B62" t="s">
-        <v>125</v>
       </c>
       <c r="C62" t="s">
         <v>40</v>
       </c>
       <c r="D62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E62" t="s">
         <v>80</v>
       </c>
       <c r="F62" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G62" t="s">
         <v>45</v>
@@ -6409,27 +6409,27 @@
         <v>4</v>
       </c>
       <c r="AK62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="63" spans="1:37">
       <c r="A63" t="s">
+        <v>123</v>
+      </c>
+      <c r="B63" t="s">
         <v>124</v>
-      </c>
-      <c r="B63" t="s">
-        <v>125</v>
       </c>
       <c r="C63" t="s">
         <v>40</v>
       </c>
       <c r="D63" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E63" t="s">
         <v>42</v>
       </c>
       <c r="F63" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G63" t="s">
         <v>45</v>
@@ -6444,28 +6444,28 @@
         <v>47</v>
       </c>
       <c r="L63" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M63" t="s">
         <v>44</v>
       </c>
       <c r="N63" t="s">
+        <v>95</v>
+      </c>
+      <c r="O63" t="s">
+        <v>95</v>
+      </c>
+      <c r="P63" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>48</v>
+      </c>
+      <c r="T63" t="s">
         <v>96</v>
       </c>
-      <c r="O63" t="s">
+      <c r="U63" t="s">
         <v>96</v>
-      </c>
-      <c r="P63" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q63" t="s">
-        <v>48</v>
-      </c>
-      <c r="T63" t="s">
-        <v>97</v>
-      </c>
-      <c r="U63" t="s">
-        <v>97</v>
       </c>
       <c r="V63" t="s">
         <v>51</v>
@@ -6477,7 +6477,7 @@
         <v>53</v>
       </c>
       <c r="AA63" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AB63" t="s">
         <v>51</v>
@@ -6507,27 +6507,27 @@
         <v>1</v>
       </c>
       <c r="AK63" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="64" spans="1:37">
       <c r="A64" t="s">
+        <v>123</v>
+      </c>
+      <c r="B64" t="s">
         <v>124</v>
-      </c>
-      <c r="B64" t="s">
-        <v>125</v>
       </c>
       <c r="C64" t="s">
         <v>40</v>
       </c>
       <c r="D64" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E64" t="s">
         <v>57</v>
       </c>
       <c r="F64" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G64" t="s">
         <v>45</v>
@@ -6607,16 +6607,16 @@
     </row>
     <row r="65" spans="1:37">
       <c r="A65" t="s">
+        <v>123</v>
+      </c>
+      <c r="B65" t="s">
         <v>124</v>
-      </c>
-      <c r="B65" t="s">
-        <v>125</v>
       </c>
       <c r="C65" t="s">
         <v>40</v>
       </c>
       <c r="D65" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E65" t="s">
         <v>64</v>
@@ -6634,46 +6634,46 @@
         <v>47</v>
       </c>
       <c r="L65" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M65" t="s">
         <v>45</v>
       </c>
       <c r="N65" t="s">
+        <v>132</v>
+      </c>
+      <c r="P65" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>48</v>
+      </c>
+      <c r="T65" t="s">
+        <v>132</v>
+      </c>
+      <c r="U65" t="s">
+        <v>132</v>
+      </c>
+      <c r="V65" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z65" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA65" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB65" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC65" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD65" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE65" t="s">
         <v>133</v>
-      </c>
-      <c r="P65" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q65" t="s">
-        <v>48</v>
-      </c>
-      <c r="T65" t="s">
-        <v>133</v>
-      </c>
-      <c r="U65" t="s">
-        <v>133</v>
-      </c>
-      <c r="V65" t="s">
-        <v>51</v>
-      </c>
-      <c r="Z65" t="s">
-        <v>51</v>
-      </c>
-      <c r="AA65" t="s">
-        <v>51</v>
-      </c>
-      <c r="AB65" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC65" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD65" t="s">
-        <v>51</v>
-      </c>
-      <c r="AE65" t="s">
-        <v>134</v>
       </c>
       <c r="AF65" t="s">
         <v>51</v>
@@ -6696,13 +6696,13 @@
     </row>
     <row r="66" spans="1:37">
       <c r="A66" t="s">
+        <v>134</v>
+      </c>
+      <c r="B66" t="s">
         <v>135</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>136</v>
-      </c>
-      <c r="C66" t="s">
-        <v>137</v>
       </c>
       <c r="D66" t="s">
         <v>41</v>
@@ -6711,19 +6711,19 @@
         <v>42</v>
       </c>
       <c r="F66" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G66" t="s">
         <v>73</v>
       </c>
       <c r="H66" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I66" t="s">
         <v>73</v>
       </c>
       <c r="J66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K66" t="s">
         <v>47</v>
@@ -6732,10 +6732,10 @@
         <v>88</v>
       </c>
       <c r="M66" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N66" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O66" t="s">
         <v>73</v>
@@ -6747,13 +6747,13 @@
         <v>48</v>
       </c>
       <c r="S66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V66" t="s">
         <v>51</v>
       </c>
       <c r="X66" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Z66" t="s">
         <v>53</v>
@@ -6789,18 +6789,18 @@
         <v>0</v>
       </c>
       <c r="AK66" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="67" spans="1:37">
       <c r="A67" t="s">
+        <v>134</v>
+      </c>
+      <c r="B67" t="s">
         <v>135</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>136</v>
-      </c>
-      <c r="C67" t="s">
-        <v>137</v>
       </c>
       <c r="D67" t="s">
         <v>56</v>
@@ -6809,31 +6809,31 @@
         <v>57</v>
       </c>
       <c r="F67" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G67" t="s">
         <v>73</v>
       </c>
       <c r="H67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I67" t="s">
         <v>73</v>
       </c>
       <c r="J67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K67" t="s">
         <v>47</v>
       </c>
       <c r="L67" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N67" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O67" t="s">
         <v>88</v>
@@ -6845,7 +6845,7 @@
         <v>48</v>
       </c>
       <c r="S67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V67" t="s">
         <v>51</v>
@@ -6884,18 +6884,18 @@
         <v>0</v>
       </c>
       <c r="AK67" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="68" spans="1:37">
       <c r="A68" t="s">
+        <v>134</v>
+      </c>
+      <c r="B68" t="s">
         <v>135</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>136</v>
-      </c>
-      <c r="C68" t="s">
-        <v>137</v>
       </c>
       <c r="D68" t="s">
         <v>63</v>
@@ -6919,7 +6919,7 @@
         <v>87</v>
       </c>
       <c r="M68" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N68" t="s">
         <v>144</v>
@@ -6978,13 +6978,13 @@
     </row>
     <row r="69" spans="1:37">
       <c r="A69" t="s">
+        <v>134</v>
+      </c>
+      <c r="B69" t="s">
         <v>135</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>136</v>
-      </c>
-      <c r="C69" t="s">
-        <v>137</v>
       </c>
       <c r="D69" t="s">
         <v>69</v>
@@ -6993,19 +6993,19 @@
         <v>70</v>
       </c>
       <c r="F69" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G69" t="s">
         <v>73</v>
       </c>
       <c r="H69" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I69" t="s">
         <v>73</v>
       </c>
       <c r="J69" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K69" t="s">
         <v>47</v>
@@ -7014,7 +7014,7 @@
         <v>74</v>
       </c>
       <c r="M69" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N69" t="s">
         <v>146</v>
@@ -7029,7 +7029,7 @@
         <v>48</v>
       </c>
       <c r="S69" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V69" t="s">
         <v>51</v>
@@ -7071,18 +7071,18 @@
         <v>0</v>
       </c>
       <c r="AK69" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="70" spans="1:37">
       <c r="A70" t="s">
+        <v>134</v>
+      </c>
+      <c r="B70" t="s">
         <v>135</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>136</v>
-      </c>
-      <c r="C70" t="s">
-        <v>137</v>
       </c>
       <c r="D70" t="s">
         <v>71</v>
@@ -7091,19 +7091,19 @@
         <v>72</v>
       </c>
       <c r="F70" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G70" t="s">
         <v>73</v>
       </c>
       <c r="H70" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I70" t="s">
         <v>73</v>
       </c>
       <c r="J70" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K70" t="s">
         <v>47</v>
@@ -7112,7 +7112,7 @@
         <v>48</v>
       </c>
       <c r="M70" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="O70" t="s">
         <v>148</v>
@@ -7124,7 +7124,7 @@
         <v>48</v>
       </c>
       <c r="S70" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V70" t="s">
         <v>51</v>
@@ -7171,13 +7171,13 @@
     </row>
     <row r="71" spans="1:37">
       <c r="A71" t="s">
+        <v>134</v>
+      </c>
+      <c r="B71" t="s">
         <v>135</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>136</v>
-      </c>
-      <c r="C71" t="s">
-        <v>137</v>
       </c>
       <c r="D71" t="s">
         <v>77</v>
@@ -7186,19 +7186,19 @@
         <v>78</v>
       </c>
       <c r="F71" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G71" t="s">
         <v>73</v>
       </c>
       <c r="H71" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I71" t="s">
         <v>73</v>
       </c>
       <c r="J71" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K71" t="s">
         <v>47</v>
@@ -7219,7 +7219,7 @@
         <v>48</v>
       </c>
       <c r="S71" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V71" t="s">
         <v>51</v>
@@ -7266,13 +7266,13 @@
     </row>
     <row r="72" spans="1:37">
       <c r="A72" t="s">
+        <v>134</v>
+      </c>
+      <c r="B72" t="s">
         <v>135</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>136</v>
-      </c>
-      <c r="C72" t="s">
-        <v>137</v>
       </c>
       <c r="D72" t="s">
         <v>79</v>
@@ -7281,19 +7281,19 @@
         <v>80</v>
       </c>
       <c r="F72" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G72" t="s">
         <v>73</v>
       </c>
       <c r="H72" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I72" t="s">
         <v>73</v>
       </c>
       <c r="J72" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K72" t="s">
         <v>47</v>
@@ -7317,7 +7317,7 @@
         <v>48</v>
       </c>
       <c r="S72" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V72" t="s">
         <v>51</v>
@@ -7359,18 +7359,18 @@
         <v>0</v>
       </c>
       <c r="AK72" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73" spans="1:37">
       <c r="A73" t="s">
+        <v>134</v>
+      </c>
+      <c r="B73" t="s">
         <v>135</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>136</v>
-      </c>
-      <c r="C73" t="s">
-        <v>137</v>
       </c>
       <c r="D73" t="s">
         <v>81</v>
@@ -7379,19 +7379,19 @@
         <v>42</v>
       </c>
       <c r="F73" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G73" t="s">
         <v>73</v>
       </c>
       <c r="H73" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I73" t="s">
         <v>73</v>
       </c>
       <c r="J73" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K73" t="s">
         <v>47</v>
@@ -7403,7 +7403,7 @@
         <v>152</v>
       </c>
       <c r="N73" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O73" t="s">
         <v>88</v>
@@ -7415,7 +7415,7 @@
         <v>48</v>
       </c>
       <c r="S73" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V73" t="s">
         <v>51</v>
@@ -7454,18 +7454,18 @@
         <v>0</v>
       </c>
       <c r="AK73" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" spans="1:37">
       <c r="A74" t="s">
+        <v>134</v>
+      </c>
+      <c r="B74" t="s">
         <v>135</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>136</v>
-      </c>
-      <c r="C74" t="s">
-        <v>137</v>
       </c>
       <c r="D74" t="s">
         <v>85</v>
@@ -7474,19 +7474,19 @@
         <v>57</v>
       </c>
       <c r="F74" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G74" t="s">
         <v>73</v>
       </c>
       <c r="H74" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I74" t="s">
         <v>73</v>
       </c>
       <c r="J74" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K74" t="s">
         <v>47</v>
@@ -7495,7 +7495,7 @@
         <v>73</v>
       </c>
       <c r="M74" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N74" t="s">
         <v>153</v>
@@ -7510,7 +7510,7 @@
         <v>48</v>
       </c>
       <c r="S74" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V74" t="s">
         <v>51</v>
@@ -7549,21 +7549,21 @@
         <v>0</v>
       </c>
       <c r="AK74" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="75" spans="1:37">
       <c r="A75" t="s">
+        <v>134</v>
+      </c>
+      <c r="B75" t="s">
         <v>135</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>136</v>
       </c>
-      <c r="C75" t="s">
-        <v>137</v>
-      </c>
       <c r="D75" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E75" t="s">
         <v>64</v>
@@ -7587,7 +7587,7 @@
         <v>154</v>
       </c>
       <c r="N75" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P75" t="s">
         <v>48</v>
@@ -7596,10 +7596,10 @@
         <v>48</v>
       </c>
       <c r="T75" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="U75" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="V75" t="s">
         <v>51</v>
@@ -7643,34 +7643,34 @@
     </row>
     <row r="76" spans="1:37">
       <c r="A76" t="s">
+        <v>134</v>
+      </c>
+      <c r="B76" t="s">
         <v>135</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>136</v>
       </c>
-      <c r="C76" t="s">
-        <v>137</v>
-      </c>
       <c r="D76" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E76" t="s">
         <v>70</v>
       </c>
       <c r="F76" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G76" t="s">
         <v>73</v>
       </c>
       <c r="H76" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I76" t="s">
         <v>73</v>
       </c>
       <c r="J76" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K76" t="s">
         <v>47</v>
@@ -7691,7 +7691,7 @@
         <v>48</v>
       </c>
       <c r="S76" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V76" t="s">
         <v>51</v>
@@ -7738,34 +7738,34 @@
     </row>
     <row r="77" spans="1:37">
       <c r="A77" t="s">
+        <v>134</v>
+      </c>
+      <c r="B77" t="s">
         <v>135</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>136</v>
       </c>
-      <c r="C77" t="s">
-        <v>137</v>
-      </c>
       <c r="D77" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E77" t="s">
         <v>72</v>
       </c>
       <c r="F77" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G77" t="s">
         <v>73</v>
       </c>
       <c r="H77" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I77" t="s">
         <v>73</v>
       </c>
       <c r="J77" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K77" t="s">
         <v>47</v>
@@ -7786,7 +7786,7 @@
         <v>48</v>
       </c>
       <c r="S77" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V77" t="s">
         <v>51</v>
@@ -7833,34 +7833,34 @@
     </row>
     <row r="78" spans="1:37">
       <c r="A78" t="s">
+        <v>134</v>
+      </c>
+      <c r="B78" t="s">
         <v>135</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>136</v>
       </c>
-      <c r="C78" t="s">
-        <v>137</v>
-      </c>
       <c r="D78" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E78" t="s">
         <v>78</v>
       </c>
       <c r="F78" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G78" t="s">
         <v>73</v>
       </c>
       <c r="H78" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I78" t="s">
         <v>73</v>
       </c>
       <c r="J78" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K78" t="s">
         <v>47</v>
@@ -7881,7 +7881,7 @@
         <v>48</v>
       </c>
       <c r="S78" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V78" t="s">
         <v>51</v>
@@ -7928,34 +7928,34 @@
     </row>
     <row r="79" spans="1:37">
       <c r="A79" t="s">
+        <v>134</v>
+      </c>
+      <c r="B79" t="s">
         <v>135</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C79" t="s">
         <v>136</v>
       </c>
-      <c r="C79" t="s">
-        <v>137</v>
-      </c>
       <c r="D79" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E79" t="s">
         <v>80</v>
       </c>
       <c r="F79" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G79" t="s">
         <v>73</v>
       </c>
       <c r="H79" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I79" t="s">
         <v>73</v>
       </c>
       <c r="J79" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K79" t="s">
         <v>47</v>
@@ -7976,7 +7976,7 @@
         <v>48</v>
       </c>
       <c r="S79" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V79" t="s">
         <v>51</v>
@@ -8023,34 +8023,34 @@
     </row>
     <row r="80" spans="1:37">
       <c r="A80" t="s">
+        <v>134</v>
+      </c>
+      <c r="B80" t="s">
         <v>135</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>136</v>
       </c>
-      <c r="C80" t="s">
-        <v>137</v>
-      </c>
       <c r="D80" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E80" t="s">
         <v>42</v>
       </c>
       <c r="F80" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G80" t="s">
         <v>73</v>
       </c>
       <c r="H80" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I80" t="s">
         <v>73</v>
       </c>
       <c r="J80" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K80" t="s">
         <v>47</v>
@@ -8071,7 +8071,7 @@
         <v>48</v>
       </c>
       <c r="S80" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V80" t="s">
         <v>51</v>
@@ -8118,34 +8118,34 @@
     </row>
     <row r="81" spans="1:37">
       <c r="A81" t="s">
+        <v>134</v>
+      </c>
+      <c r="B81" t="s">
         <v>135</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>136</v>
       </c>
-      <c r="C81" t="s">
-        <v>137</v>
-      </c>
       <c r="D81" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E81" t="s">
         <v>57</v>
       </c>
       <c r="F81" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G81" t="s">
         <v>73</v>
       </c>
       <c r="H81" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I81" t="s">
         <v>73</v>
       </c>
       <c r="J81" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K81" t="s">
         <v>47</v>
@@ -8154,7 +8154,7 @@
         <v>73</v>
       </c>
       <c r="M81" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N81" t="s">
         <v>153</v>
@@ -8169,7 +8169,7 @@
         <v>48</v>
       </c>
       <c r="S81" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V81" t="s">
         <v>51</v>
@@ -8208,21 +8208,21 @@
         <v>0</v>
       </c>
       <c r="AK81" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="82" spans="1:37">
       <c r="A82" t="s">
+        <v>134</v>
+      </c>
+      <c r="B82" t="s">
         <v>135</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
         <v>136</v>
       </c>
-      <c r="C82" t="s">
-        <v>137</v>
-      </c>
       <c r="D82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E82" t="s">
         <v>64</v>
@@ -8243,7 +8243,7 @@
         <v>73</v>
       </c>
       <c r="M82" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N82" t="s">
         <v>153</v>
@@ -8302,34 +8302,34 @@
     </row>
     <row r="83" spans="1:37">
       <c r="A83" t="s">
+        <v>134</v>
+      </c>
+      <c r="B83" t="s">
         <v>135</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>136</v>
       </c>
-      <c r="C83" t="s">
-        <v>137</v>
-      </c>
       <c r="D83" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E83" t="s">
         <v>70</v>
       </c>
       <c r="F83" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G83" t="s">
         <v>73</v>
       </c>
       <c r="H83" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I83" t="s">
         <v>73</v>
       </c>
       <c r="J83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K83" t="s">
         <v>47</v>
@@ -8338,7 +8338,7 @@
         <v>73</v>
       </c>
       <c r="M83" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N83" t="s">
         <v>153</v>
@@ -8353,7 +8353,7 @@
         <v>48</v>
       </c>
       <c r="S83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V83" t="s">
         <v>51</v>
@@ -8392,39 +8392,39 @@
         <v>0</v>
       </c>
       <c r="AK83" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="84" spans="1:37">
       <c r="A84" t="s">
+        <v>134</v>
+      </c>
+      <c r="B84" t="s">
         <v>135</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>136</v>
       </c>
-      <c r="C84" t="s">
-        <v>137</v>
-      </c>
       <c r="D84" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E84" t="s">
         <v>72</v>
       </c>
       <c r="F84" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G84" t="s">
         <v>73</v>
       </c>
       <c r="H84" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I84" t="s">
         <v>73</v>
       </c>
       <c r="J84" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K84" t="s">
         <v>47</v>
@@ -8433,7 +8433,7 @@
         <v>73</v>
       </c>
       <c r="M84" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N84" t="s">
         <v>153</v>
@@ -8448,7 +8448,7 @@
         <v>48</v>
       </c>
       <c r="S84" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V84" t="s">
         <v>51</v>
@@ -8487,39 +8487,39 @@
         <v>0</v>
       </c>
       <c r="AK84" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="85" spans="1:37">
       <c r="A85" t="s">
+        <v>134</v>
+      </c>
+      <c r="B85" t="s">
         <v>135</v>
       </c>
-      <c r="B85" t="s">
+      <c r="C85" t="s">
         <v>136</v>
       </c>
-      <c r="C85" t="s">
-        <v>137</v>
-      </c>
       <c r="D85" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E85" t="s">
         <v>78</v>
       </c>
       <c r="F85" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G85" t="s">
         <v>73</v>
       </c>
       <c r="H85" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I85" t="s">
         <v>73</v>
       </c>
       <c r="J85" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K85" t="s">
         <v>47</v>
@@ -8528,7 +8528,7 @@
         <v>73</v>
       </c>
       <c r="M85" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N85" t="s">
         <v>153</v>
@@ -8543,7 +8543,7 @@
         <v>48</v>
       </c>
       <c r="S85" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V85" t="s">
         <v>51</v>
@@ -8582,39 +8582,39 @@
         <v>0</v>
       </c>
       <c r="AK85" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="86" spans="1:37">
       <c r="A86" t="s">
+        <v>134</v>
+      </c>
+      <c r="B86" t="s">
         <v>135</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C86" t="s">
         <v>136</v>
       </c>
-      <c r="C86" t="s">
-        <v>137</v>
-      </c>
       <c r="D86" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E86" t="s">
         <v>80</v>
       </c>
       <c r="F86" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G86" t="s">
         <v>73</v>
       </c>
       <c r="H86" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I86" t="s">
         <v>73</v>
       </c>
       <c r="J86" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K86" t="s">
         <v>47</v>
@@ -8623,7 +8623,7 @@
         <v>73</v>
       </c>
       <c r="M86" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N86" t="s">
         <v>153</v>
@@ -8638,7 +8638,7 @@
         <v>48</v>
       </c>
       <c r="S86" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V86" t="s">
         <v>51</v>
@@ -8677,39 +8677,39 @@
         <v>0</v>
       </c>
       <c r="AK86" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="87" spans="1:37">
       <c r="A87" t="s">
+        <v>134</v>
+      </c>
+      <c r="B87" t="s">
         <v>135</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C87" t="s">
         <v>136</v>
       </c>
-      <c r="C87" t="s">
-        <v>137</v>
-      </c>
       <c r="D87" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E87" t="s">
         <v>42</v>
       </c>
       <c r="F87" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G87" t="s">
         <v>73</v>
       </c>
       <c r="H87" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I87" t="s">
         <v>73</v>
       </c>
       <c r="J87" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K87" t="s">
         <v>47</v>
@@ -8718,7 +8718,7 @@
         <v>73</v>
       </c>
       <c r="M87" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N87" t="s">
         <v>153</v>
@@ -8733,7 +8733,7 @@
         <v>48</v>
       </c>
       <c r="S87" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V87" t="s">
         <v>51</v>
@@ -8772,39 +8772,39 @@
         <v>0</v>
       </c>
       <c r="AK87" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="88" spans="1:37">
       <c r="A88" t="s">
+        <v>134</v>
+      </c>
+      <c r="B88" t="s">
         <v>135</v>
       </c>
-      <c r="B88" t="s">
+      <c r="C88" t="s">
         <v>136</v>
       </c>
-      <c r="C88" t="s">
-        <v>137</v>
-      </c>
       <c r="D88" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E88" t="s">
         <v>57</v>
       </c>
       <c r="F88" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G88" t="s">
         <v>73</v>
       </c>
       <c r="H88" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I88" t="s">
         <v>73</v>
       </c>
       <c r="J88" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K88" t="s">
         <v>47</v>
@@ -8813,7 +8813,7 @@
         <v>73</v>
       </c>
       <c r="M88" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N88" t="s">
         <v>153</v>
@@ -8828,7 +8828,7 @@
         <v>48</v>
       </c>
       <c r="S88" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V88" t="s">
         <v>51</v>
@@ -8867,21 +8867,21 @@
         <v>0</v>
       </c>
       <c r="AK88" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="89" spans="1:37">
       <c r="A89" t="s">
+        <v>134</v>
+      </c>
+      <c r="B89" t="s">
         <v>135</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>136</v>
       </c>
-      <c r="C89" t="s">
-        <v>137</v>
-      </c>
       <c r="D89" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E89" t="s">
         <v>64</v>
@@ -8902,7 +8902,7 @@
         <v>73</v>
       </c>
       <c r="M89" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N89" t="s">
         <v>153</v>
@@ -8961,34 +8961,34 @@
     </row>
     <row r="90" spans="1:37">
       <c r="A90" t="s">
+        <v>134</v>
+      </c>
+      <c r="B90" t="s">
         <v>135</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C90" t="s">
         <v>136</v>
       </c>
-      <c r="C90" t="s">
-        <v>137</v>
-      </c>
       <c r="D90" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E90" t="s">
         <v>70</v>
       </c>
       <c r="F90" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G90" t="s">
         <v>73</v>
       </c>
       <c r="H90" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I90" t="s">
         <v>73</v>
       </c>
       <c r="J90" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K90" t="s">
         <v>47</v>
@@ -9009,7 +9009,7 @@
         <v>48</v>
       </c>
       <c r="S90" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V90" t="s">
         <v>51</v>
@@ -9056,34 +9056,34 @@
     </row>
     <row r="91" spans="1:37">
       <c r="A91" t="s">
+        <v>134</v>
+      </c>
+      <c r="B91" t="s">
         <v>135</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C91" t="s">
         <v>136</v>
       </c>
-      <c r="C91" t="s">
-        <v>137</v>
-      </c>
       <c r="D91" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E91" t="s">
         <v>72</v>
       </c>
       <c r="F91" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G91" t="s">
         <v>73</v>
       </c>
       <c r="H91" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I91" t="s">
         <v>73</v>
       </c>
       <c r="J91" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K91" t="s">
         <v>47</v>
@@ -9092,7 +9092,7 @@
         <v>73</v>
       </c>
       <c r="M91" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N91" t="s">
         <v>153</v>
@@ -9107,7 +9107,7 @@
         <v>48</v>
       </c>
       <c r="S91" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V91" t="s">
         <v>51</v>
@@ -9146,39 +9146,39 @@
         <v>0</v>
       </c>
       <c r="AK91" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="92" spans="1:37">
       <c r="A92" t="s">
+        <v>134</v>
+      </c>
+      <c r="B92" t="s">
         <v>135</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>136</v>
       </c>
-      <c r="C92" t="s">
-        <v>137</v>
-      </c>
       <c r="D92" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E92" t="s">
         <v>78</v>
       </c>
       <c r="F92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G92" t="s">
         <v>73</v>
       </c>
       <c r="H92" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I92" t="s">
         <v>73</v>
       </c>
       <c r="J92" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K92" t="s">
         <v>47</v>
@@ -9187,7 +9187,7 @@
         <v>73</v>
       </c>
       <c r="M92" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N92" t="s">
         <v>153</v>
@@ -9202,7 +9202,7 @@
         <v>48</v>
       </c>
       <c r="S92" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V92" t="s">
         <v>51</v>
@@ -9241,39 +9241,39 @@
         <v>0</v>
       </c>
       <c r="AK92" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="93" spans="1:37">
       <c r="A93" t="s">
+        <v>134</v>
+      </c>
+      <c r="B93" t="s">
         <v>135</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
         <v>136</v>
       </c>
-      <c r="C93" t="s">
-        <v>137</v>
-      </c>
       <c r="D93" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E93" t="s">
         <v>80</v>
       </c>
       <c r="F93" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G93" t="s">
         <v>73</v>
       </c>
       <c r="H93" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I93" t="s">
         <v>73</v>
       </c>
       <c r="J93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K93" t="s">
         <v>47</v>
@@ -9282,7 +9282,7 @@
         <v>73</v>
       </c>
       <c r="M93" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N93" t="s">
         <v>153</v>
@@ -9297,7 +9297,7 @@
         <v>48</v>
       </c>
       <c r="S93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V93" t="s">
         <v>51</v>
@@ -9336,39 +9336,39 @@
         <v>0</v>
       </c>
       <c r="AK93" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="94" spans="1:37">
       <c r="A94" t="s">
+        <v>134</v>
+      </c>
+      <c r="B94" t="s">
         <v>135</v>
       </c>
-      <c r="B94" t="s">
+      <c r="C94" t="s">
         <v>136</v>
       </c>
-      <c r="C94" t="s">
-        <v>137</v>
-      </c>
       <c r="D94" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E94" t="s">
         <v>42</v>
       </c>
       <c r="F94" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G94" t="s">
         <v>73</v>
       </c>
       <c r="H94" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I94" t="s">
         <v>73</v>
       </c>
       <c r="J94" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K94" t="s">
         <v>47</v>
@@ -9386,7 +9386,7 @@
         <v>48</v>
       </c>
       <c r="S94" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V94" t="s">
         <v>51</v>
@@ -9433,34 +9433,34 @@
     </row>
     <row r="95" spans="1:37">
       <c r="A95" t="s">
+        <v>134</v>
+      </c>
+      <c r="B95" t="s">
         <v>135</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C95" t="s">
         <v>136</v>
       </c>
-      <c r="C95" t="s">
-        <v>137</v>
-      </c>
       <c r="D95" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E95" t="s">
         <v>57</v>
       </c>
       <c r="F95" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G95" t="s">
         <v>73</v>
       </c>
       <c r="H95" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I95" t="s">
         <v>73</v>
       </c>
       <c r="J95" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K95" t="s">
         <v>47</v>
@@ -9481,7 +9481,7 @@
         <v>48</v>
       </c>
       <c r="S95" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V95" t="s">
         <v>51</v>
@@ -9528,16 +9528,16 @@
     </row>
     <row r="96" spans="1:37">
       <c r="A96" t="s">
+        <v>134</v>
+      </c>
+      <c r="B96" t="s">
         <v>135</v>
       </c>
-      <c r="B96" t="s">
+      <c r="C96" t="s">
         <v>136</v>
       </c>
-      <c r="C96" t="s">
-        <v>137</v>
-      </c>
       <c r="D96" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E96" t="s">
         <v>64</v>
@@ -9555,7 +9555,7 @@
         <v>47</v>
       </c>
       <c r="L96" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="M96" t="s">
         <v>48</v>

</xml_diff>